<commit_message>
Added stragglers and refine image alignment / background
</commit_message>
<xml_diff>
--- a/Elle's Surprise Bday Collage 2026 (Responses).xlsx
+++ b/Elle's Surprise Bday Collage 2026 (Responses).xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\devin\Documents\Dev\elles-birthday-collage\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97F6E80B-D07D-4135-BBAC-E35C7F407768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Form Responses 1" sheetId="1" r:id="rId5"/>
+    <sheet name="Form Responses 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="116">
   <si>
     <t>Timestamp</t>
   </si>
@@ -340,28 +349,57 @@
   <si>
     <t>it's amazing how one person can be so energetic and then also sleep through anything. versatile like a futon! but also croissaints were taken :'(</t>
   </si>
+  <si>
+    <t>Sherry</t>
+  </si>
+  <si>
+    <t>Bright yellow door</t>
+  </si>
+  <si>
+    <t>Portal to different worlds and people. Welcoming!</t>
+  </si>
+  <si>
+    <t>Katie Lee</t>
+  </si>
+  <si>
+    <t>Laying a line of sparklers into the unknown</t>
+  </si>
+  <si>
+    <t>It has so much brightness and follows a path that you might not expect, but it gives joy and confidence to those around and reminds you that the journey is worthwhile.</t>
+  </si>
+  <si>
+    <t>Nupoor (aka the real korean of the family)</t>
+  </si>
+  <si>
+    <t>crabs🦀</t>
+  </si>
+  <si>
+    <t>Claw Daddy was one of the my favorite moments with Elle (and i guess Devin was there too) and of 2025. We spent a few hours yapping about random stuff and breaking open crab legs together but it was one of the first times we actually spent 1-1 time.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="m/d/yyyy h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Roboto"/>
     </font>
@@ -371,76 +409,41 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF5B3F86"/>
-          <bgColor rgb="FF5B3F86"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8F9FA"/>
-          <bgColor rgb="FFF8F9FA"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <border>
         <left style="thin">
@@ -457,41 +460,65 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8F9FA"/>
+          <bgColor rgb="FFF8F9FA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF5B3F86"/>
+          <bgColor rgb="FF5B3F86"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="4" pivot="0" name="Form Responses 1-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    <tableStyle name="Form Responses 1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
+      <tableStyleElement type="headerRow" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="secondRowStripe" dxfId="1"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E30" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:E33">
   <tableColumns count="5">
-    <tableColumn name="Timestamp" id="1"/>
-    <tableColumn name="Who are you? (name as you want it to appear to Elle)" id="2"/>
-    <tableColumn name="What object (physical or metaphysical) reminds you of Elle?" id="3"/>
-    <tableColumn name="Why (don't think too much - keep it short and spontaneous like Elle) - 1 to 2 sentences is fine" id="4"/>
-    <tableColumn name="If you have an image of the specific object in mind, attach it here. Totally optional, me and Claude will find the object if not._x000a__x000a_Insert the image URL below" id="5"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Timestamp"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Who are you? (name as you want it to appear to Elle)"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="What object (physical or metaphysical) reminds you of Elle?"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Why (don't think too much - keep it short and spontaneous like Elle) - 1 to 2 sentences is fine"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="If you have an image of the specific object in mind, attach it here. Totally optional, me and Claude will find the object if not._x000a__x000a_Insert the image URL below"/>
   </tableColumns>
-  <tableStyleInfo name="Form Responses 1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Form Responses 1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -681,22 +708,25 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:E33"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="18.88"/>
-    <col customWidth="1" min="2" max="5" width="37.63"/>
-    <col customWidth="1" min="6" max="11" width="18.88"/>
+    <col min="1" max="1" width="18.85546875" customWidth="1"/>
+    <col min="2" max="5" width="37.5703125" customWidth="1"/>
+    <col min="6" max="11" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1">
+    <row r="1" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -713,9 +743,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" ht="22.5" customHeight="1">
+    <row r="2" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
-        <v>46144.20360420139</v>
+        <v>46144.203604201393</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>5</v>
@@ -726,9 +756,9 @@
       <c r="D2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="4"/>
-    </row>
-    <row r="3" ht="22.5" customHeight="1">
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>46144.273667974536</v>
       </c>
@@ -741,11 +771,11 @@
       <c r="D3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="4"/>
-    </row>
-    <row r="4" ht="22.5" customHeight="1">
+      <c r="E3" s="3"/>
+    </row>
+    <row r="4" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
-        <v>46144.27482868056</v>
+        <v>46144.274828680558</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>11</v>
@@ -760,9 +790,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" ht="22.5" customHeight="1">
+    <row r="5" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
-        <v>46144.28715230324</v>
+        <v>46144.287152303237</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>15</v>
@@ -773,13 +803,13 @@
       <c r="D5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" ht="22.5" customHeight="1">
+    <row r="6" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>46144.4187140162</v>
+        <v>46144.418714016203</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>19</v>
@@ -790,11 +820,11 @@
       <c r="D6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="4"/>
-    </row>
-    <row r="7" ht="22.5" customHeight="1">
+      <c r="E6" s="3"/>
+    </row>
+    <row r="7" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>46144.44578913195</v>
+        <v>46144.445789131947</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>22</v>
@@ -809,9 +839,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" ht="22.5" customHeight="1">
+    <row r="8" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>46144.49250765046</v>
+        <v>46144.492507650459</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>26</v>
@@ -822,11 +852,11 @@
       <c r="D8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" ht="22.5" customHeight="1">
+    <row r="9" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>46144.75987469907</v>
       </c>
@@ -843,9 +873,9 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1">
+    <row r="10" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>46144.9209666088</v>
+        <v>46144.920966608799</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>34</v>
@@ -860,9 +890,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" ht="22.5" customHeight="1">
+    <row r="11" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>46145.52800828704</v>
+        <v>46145.528008287038</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>38</v>
@@ -873,11 +903,11 @@
       <c r="D11" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E11" s="4"/>
-    </row>
-    <row r="12" ht="22.5" customHeight="1">
+      <c r="E11" s="3"/>
+    </row>
+    <row r="12" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>46145.57875810185</v>
+        <v>46145.578758101852</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>41</v>
@@ -888,13 +918,13 @@
       <c r="D12" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="13" ht="22.5" customHeight="1">
+    <row r="13" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>46145.76790420139</v>
+        <v>46145.767904201392</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>45</v>
@@ -905,11 +935,11 @@
       <c r="D13" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="4" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="14" ht="22.5" customHeight="1">
+    <row r="14" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>46146.393232372684</v>
       </c>
@@ -922,9 +952,9 @@
       <c r="D14" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E14" s="4"/>
-    </row>
-    <row r="15" ht="22.5" customHeight="1">
+      <c r="E14" s="3"/>
+    </row>
+    <row r="15" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>46146.417781909724</v>
       </c>
@@ -941,9 +971,9 @@
         <v>55</v>
       </c>
     </row>
-    <row r="16" ht="22.5" customHeight="1">
+    <row r="16" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>46146.46748278935</v>
+        <v>46146.467482789347</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>56</v>
@@ -958,9 +988,9 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" ht="22.5" customHeight="1">
+    <row r="17" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>46146.51733920139</v>
+        <v>46146.517339201389</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>60</v>
@@ -971,11 +1001,11 @@
       <c r="D17" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="18" ht="22.5" customHeight="1">
+    <row r="18" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>46146.65069800926</v>
       </c>
@@ -988,13 +1018,13 @@
       <c r="D18" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E18" s="4" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="19" ht="22.5" customHeight="1">
+    <row r="19" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>46146.65363863426</v>
+        <v>46146.653638634263</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>64</v>
@@ -1005,11 +1035,11 @@
       <c r="D19" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E19" s="4"/>
-    </row>
-    <row r="20" ht="22.5" customHeight="1">
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>46146.69468398148</v>
+        <v>46146.694683981477</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>70</v>
@@ -1020,11 +1050,11 @@
       <c r="D20" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="E20" s="4"/>
-    </row>
-    <row r="21" ht="22.5" customHeight="1">
+      <c r="E20" s="3"/>
+    </row>
+    <row r="21" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>46146.73621171297</v>
+        <v>46146.736211712967</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>73</v>
@@ -1035,11 +1065,11 @@
       <c r="D21" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E21" s="4"/>
-    </row>
-    <row r="22" ht="22.5" customHeight="1">
+      <c r="E21" s="3"/>
+    </row>
+    <row r="22" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>46146.89696532408</v>
+        <v>46146.896965324078</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>76</v>
@@ -1050,9 +1080,9 @@
       <c r="D22" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E22" s="4"/>
-    </row>
-    <row r="23" ht="22.5" customHeight="1">
+      <c r="E22" s="3"/>
+    </row>
+    <row r="23" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>46147.41764590278</v>
       </c>
@@ -1065,11 +1095,11 @@
       <c r="D23" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="E23" s="4"/>
-    </row>
-    <row r="24" ht="22.5" customHeight="1">
+      <c r="E23" s="3"/>
+    </row>
+    <row r="24" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>46147.81364679398</v>
+        <v>46147.813646793977</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>82</v>
@@ -1080,11 +1110,11 @@
       <c r="D24" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="E24" s="4"/>
-    </row>
-    <row r="25" ht="22.5" customHeight="1">
+      <c r="E24" s="3"/>
+    </row>
+    <row r="25" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>46148.16904303241</v>
+        <v>46148.169043032409</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>85</v>
@@ -1095,13 +1125,13 @@
       <c r="D25" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E25" s="4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="26" ht="22.5" customHeight="1">
+    <row r="26" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>46148.19896232639</v>
+        <v>46148.198962326387</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>89</v>
@@ -1116,9 +1146,9 @@
         <v>92</v>
       </c>
     </row>
-    <row r="27" ht="22.5" customHeight="1">
+    <row r="27" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>46148.3332995949</v>
+        <v>46148.333299594902</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>93</v>
@@ -1133,7 +1163,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="28" ht="22.5" customHeight="1">
+    <row r="28" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>46148.338139872685</v>
       </c>
@@ -1146,11 +1176,11 @@
       <c r="D28" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="E28" s="5" t="s">
+      <c r="E28" s="4" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="29" ht="22.5" customHeight="1">
+    <row r="29" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
         <v>46148.648405370375</v>
       </c>
@@ -1163,11 +1193,11 @@
       <c r="D29" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="E29" s="4" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="30" ht="22.5" customHeight="1">
+    <row r="30" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
         <v>46148.79182525463</v>
       </c>
@@ -1180,23 +1210,65 @@
       <c r="D30" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="E30" s="4"/>
+      <c r="E30" s="3"/>
+    </row>
+    <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="5">
+        <v>46148.97760416667</v>
+      </c>
+      <c r="B31" t="s">
+        <v>107</v>
+      </c>
+      <c r="C31" t="s">
+        <v>108</v>
+      </c>
+      <c r="D31" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="5">
+        <v>46149.493645833332</v>
+      </c>
+      <c r="B32" t="s">
+        <v>110</v>
+      </c>
+      <c r="C32" t="s">
+        <v>111</v>
+      </c>
+      <c r="D32" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="5">
+        <v>46149.595104166663</v>
+      </c>
+      <c r="B33" t="s">
+        <v>113</v>
+      </c>
+      <c r="C33" t="s">
+        <v>114</v>
+      </c>
+      <c r="D33" t="s">
+        <v>115</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="E5"/>
-    <hyperlink r:id="rId2" ref="E8"/>
-    <hyperlink r:id="rId3" ref="E12"/>
-    <hyperlink r:id="rId4" ref="E13"/>
-    <hyperlink r:id="rId5" ref="E17"/>
-    <hyperlink r:id="rId6" ref="E18"/>
-    <hyperlink r:id="rId7" ref="E25"/>
-    <hyperlink r:id="rId8" ref="E28"/>
-    <hyperlink r:id="rId9" ref="E29"/>
+    <hyperlink ref="E5" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="E8" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="E12" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="E13" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="E17" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="E18" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="E25" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="E28" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="E29" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
   </hyperlinks>
-  <drawing r:id="rId10"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId12"/>
+    <tablePart r:id="rId10"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>